<commit_message>
Fix Sugar News editorial validation
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-23.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-23.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -513,29 +513,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 ChiniMandi报道：El Niño seen boosting Brazil’s sugarcane crop despite harvest delays。来源：ChiniMandi（https://news.google.com/rss/articles/CBMimwFBVV95cUxPRjB6ZU43QTRKS2JCSGRFTUtQYTJyMnd0U05lSkdTdUJpT1lkZjJDeUJ3RWFVc0JsWWt6RzFhX0Q4RVBBR18zLTVJTHdvY0FycjdiakJmMzF3Q0VERlNsSFpBdlQxOVduR2pTN1VoSzBuZUpua0s0SnRWdVJ5cFhuM1dEYnJhNzNISm5zX1lUUHRzTno4dDI4aXpYTQ?oc=5）</t>
+          <t>ChiniMandi称，El Niño可能改善巴西部分甘蔗产区作物表现，但收割延迟仍扰动压榨节奏。单产改善有利于增加糖料供应，收割延后则可能推迟糖产量释放，短期影响偏中性。来源：ChiniMandi（https://news.google.com/rss/articles/CBMimwFBVV95cUxPRjB6ZU43QTRKS2JCSGRFTUtQYTJyMnd0U05lSkdTdUJpT1lkZjJDeUJ3RWFVc0JsWWt6RzFhX0Q4RVBBR18zLTVJTHdvY0FycjdiakJmMzF3Q0VERlNsSFpBdlQxOVduR2pTN1VoSzBuZUpua0s0SnRWdVJ5cFhuM1dEYnJhNzNISm5zX1lUUHRzTno4dDI4aXpYTQ?oc=5）</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="176.35" customHeight="1" s="2">
+          <t>中性：单产和收割进度影响方向相反，短期对糖价缺乏单边驱动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="180" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>巴西</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 FBC News报道：Sugar sector faces workforce crisis。来源：FBC News（https://news.google.com/rss/articles/CBMid0FVX3lxTE9IOWM5THJtN3NIREtHQ0Rxd09ZSEtJZUxnb2J2VUtQV3hGQTBQMThzYjVGUkx0ZHpkS2s3UFVfUzYtdTNHSHNuak91VkVqSnlzS0x5T1RQY3BoT2ktbzZpazB5MnBYNUwxakpsS1NxSFRvemdSby1n?oc=5）</t>
+          <t>Latin Lawyer称，Raízen 在重组过程中将一座糖厂出售给 Adecoagro。资产转让可能改变巴西糖厂产能归属和运营效率，但短期对全国糖产量影响仍需观察。来源：Latin Lawyer（https://news.google.com/rss/articles/CBMijAFBVV95cUxPeWNVcmtMWnhqV3FzUTlma1BBUjdvdmY3MEE2cURqUEJwZVdKN2NZbnpCQk01MXlueEZVczdzS0VveDFielZQVHFlbFFkTlNYOEMwbm92VGt5SHhrR3lGSDYySGtocGJTM09YTnc5YmtVV0JmZWNLd1NDQ1ZpNmFURld5UTVSLWp5VWFXOA?oc=5）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：资产重组影响产能归属，短期供需影响尚不明确。</t>
         </is>
       </c>
     </row>
@@ -547,12 +547,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 scanx.trade报道：Davangere Sugar Company to consider fund raising via warrants。来源：scanx.trade（https://news.google.com/rss/articles/CBMiugFBVV95cUxPbW03Q01xUERweWVHVzczbU1NcmxHeVVFT2JlQVc5azB2eDlkU2xpSWZmVi1MN0VaVktMdDRmZlNhN2pJeWU3Nk04NGxZSHF1Q05NVE9SekZFNFRVckE3VW1JOGE4ZkRhM3pDUnk2em1ZcEQ3RUR5MTJqWnMzUE1PM3ZCenVNZmhCSFl3Y2JkYWxEZkZZeXh4QlNvOGg1NjhJWU95enN0U0pmNTV5cWJvRGdoRmRMUG9RTlE?oc=5）</t>
+          <t>scanx.trade称，印度 Davangere Sugar Company 将审议通过认股权证融资。若融资落地，有助于改善企业资金能力和后续糖厂运营，但短期不直接改变食糖供需。来源：scanx.trade（https://news.google.com/rss/articles/CBMiugFBVV95cUxPbW03Q01xUERweWVHVzczbU1NcmxHeVVFT2JlQVc5azB2eDlkU2xpSWZmVi1MN0VaVktMdDRmZlNhN2pJeWU3Nk04NGxZSHF1Q05NVE9SekZFNFRVckE3VW1JOGE4ZkRhM3pDUnk2em1ZcEQ3RUR5MTJqWnMzUE1PM3ZCenVNZmhCSFl3Y2JkYWxEZkZZeXh4QlNvOGg1NjhJWU95enN0U0pmNTV5cWJvRGdoRmRMUG9RTlE?oc=5）</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：企业融资改善经营弹性，但对当期供需影响有限。</t>
         </is>
       </c>
     </row>
@@ -564,12 +564,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 ChiniMandi报道：DCM Shriram honours 154 sugarcane farmers for achieving high cane yields。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiogFBVV95cUxQNzI5RmV6QWNqejNxalM0cktYNkpiRE9tTFVUMGE2Y1dUQkpIUWRMTlllNnp2TUQ4dTl1aUFoaFJ3NWVOU0VHazVTS1pLR1JzTVZMdFpSRGJwNkNFODFIbnNnbjNmUzlHTk9ZWVYxMS1GdTdQZ1pqR2VtMHUtb09tTzVUVC1HS3hCUTVTU3MtQV81YVNNcE0yR3U5LW1qYXRyQVE?oc=5）</t>
+          <t>ChiniMandi称，印度 DCM Shriram 表彰154名甘蔗高产农户，显示部分产区单产提升和种植管理改善。高单产经验推广有助于稳定后续糖料供应，对中长期糖价偏利空。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiogFBVV95cUxQNzI5RmV6QWNqejNxalM0cktYNkpiRE9tTFVUMGE2Y1dUQkpIUWRMTlllNnp2TUQ4dTl1aUFoaFJ3NWVOU0VHazVTS1pLR1JzTVZMdFpSRGJwNkNFODFIbnNnbjNmUzlHTk9ZWVYxMS1GdTdQZ1pqR2VtMHUtb09tTzVUVC1HS3hCUTVTU3MtQV81YVNNcE0yR3U5LW1qYXRyQVE?oc=5）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：甘蔗单产改善有利于提高未来糖料供应预期。</t>
         </is>
       </c>
     </row>
@@ -581,12 +581,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 ChiniMandi报道：Bihar: Sugarcane farmers adopt neem-based solution to protect crops from wild animals。来源：ChiniMandi（https://news.google.com/rss/articles/CBMisgFBVV95cUxOM3phQWFYeDJ2WTl0NGtPMGhNSVVOSHFhcEJYcUZtOGpJd1huTjNCanZhVzgxTEFSckpTcGpYNUlaMlhyTHM5WlpOUnpTZlpnYW93RFZHaHhOQ2FtMWthcVZSTklsNkNCSk5NS1dEQ1J3N3RfQ2taZnBLZjZGNFpZeklmS1c5Y3E2aXM5ZlhtTjBETkt2eWY5dzNvMkRDdWhiTlFoZjJ0eFVYUGJNLVdaSl9B?oc=5）</t>
+          <t>ChiniMandi称，比哈尔邦蔗农采用楝树制剂防护野生动物对甘蔗作物的损害。若防护措施有效，可减少田间损失并稳定甘蔗供应，短期影响仍以区域性为主。来源：ChiniMandi（https://news.google.com/rss/articles/CBMisgFBVV95cUxOM3phQWFYeDJ2WTl0NGtPMGhNSVVOSHFhcEJYcUZtOGpJd1huTjNCanZhVzgxTEFSckpTcGpYNUlaMlhyTHM5WlpOUnpTZlpnYW93RFZHaHhOQ2FtMWthcVZSTklsNkNCSk5NS1dEQ1J3N3RfQ2taZnBLZjZGNFpZeklmS1c5Y3E2aXM5ZlhtTjBETkt2eWY5dzNvMkRDdWhiTlFoZjJ0eFVYUGJNLVdaSl9B?oc=5）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：防护措施有助于降低局部损失，但对印度总体供应影响有限。</t>
         </is>
       </c>
     </row>
@@ -598,182 +598,148 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 Mongabay India报道：Rising sugarcane yields coexist with climate, water risks in semi-arid India。来源：Mongabay India（https://news.google.com/rss/articles/CBMisAFBVV95cUxPbUtLTWhsTUI0VG9lN3ZXWmNzSVB6aWtpX2NKZjcwOENxdUN4QVU4OWZIWGdnSTlHcnlSVnhZLTYtRDdVMFFlVTcxS2FwT1B3cmlmTngzZnVSWGl1NXlYT3VYMUx0WmpRMUQzNGhTNjFJS0tYRXo1RlNEcHZmSHFBSmhzWElIR3Z3Wm0wRFRCSXRPZmFuRmpBZ1NtbEdLb0o2ODhBNXNwWnJtMlUtZG1rXw?oc=5）</t>
+          <t>Mongabay India称，印度半干旱地区甘蔗单产提升的同时，仍面临气候和水资源压力。水分约束可能限制甘蔗可持续扩产，并增加未来糖料供应波动风险。来源：Mongabay India（https://news.google.com/rss/articles/CBMisAFBVV95cUxPbUtLTWhsTUI0VG9lN3ZXWmNzSVB6aWtpX2NKZjcwOENxdUN4QVU4OWZIWGdnSTlHcnlSVnhZLTYtRDdVMFFlVTcxS2FwT1B3cmlmTngzZnVSWGl1NXlYT3VYMUx0WmpRMUQzNGhTNjFJS0tYRXo1RlNEcHZmSHFBSmhzWElIR3Z3Wm0wRFRCSXRPZmFuRmpBZ1NtbEdLb0o2ODhBNXNwWnJtMlUtZG1rXw?oc=5）</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="165.9" customHeight="1" s="2">
+          <t>影响有限：报道未明确对应印度核心甘蔗主产区，需继续跟踪水资源压力是否传导至糖料供应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="180" customHeight="1" s="2">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>印度</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 FBC News报道：Cane farmers get cost relief。来源：FBC News（https://news.google.com/rss/articles/CBMibkFVX3lxTE1tSk9tQ3ZYajFRT0tuZTZBdTBKdTFaMEVwaC1hdWFmdjRtZGx4THJPVGZvNEozWW1oVzIxUUVBWlZBVWNwcWlhV0RqOXNnMHkzN2E5bmV3MkZfek0tbkxYcGNuUVc4eEE4Uk9nSERn?oc=5）</t>
+          <t>SME Futures称，印度 Allahabad 高等法院要求追究一宗持续二十年的甘蔗款案件责任。甘蔗款纠纷反映糖厂付款和蔗农现金流压力，若拖欠问题持续，可能影响后续种植积极性。来源：SME Futures（https://news.google.com/rss/articles/CBMimwFBVV95cUxPcWRaX2lqME5GZ042V092SzAyZXByMjI2N2F2R3o1bmUzUkRXSU5VOC1YYkh2MmFmQUJVTDRnN2c3WWlra21xdTlMT2M1WDJqZElKWmFHY1JkNGFMcDQteXNZOWotSjY1MThJMnVLNFE1SG0zQ1p2WktoRjVubXVsVlBCSXprLUFmYzRNbHJJOGRfd2pvaE5GTGgzNA?oc=5）</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：司法问责有助于改善付款秩序，但短期供需影响有限。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="180" customHeight="1" s="2">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>斐济</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 AOL.co.uk报道：Lord Sugar tells ITV fans 'watch out' as he calls for 'investigation' into £5 fee。来源：AOL.co.uk（https://news.google.com/rss/articles/CBMie0FVX3lxTE0ybzBOd01uVTJQdGVTc000aVNtb0Z1OGpwcjhVWFEtOFZ1WHgyUDdnYVYydnpCTi1FVUY1THhNbHhwTWlDNTUxYm1ZSGJoZkwzUVNSdFU0bWRZNHdSNWJ5d1BYeXR2V3NXdHBrVXVkQTBiQVNwYjNhaG9jRQ?oc=5）</t>
+          <t>FBC News称，斐济糖业部门面临劳动力短缺压力，甘蔗收割和糖厂运行可能受到影响。若砍蔗工供应不足持续，甘蔗入榨节奏和当季产量释放可能放慢。来源：FBC News（https://news.google.com/rss/articles/CBMid0FVX3lxTE9IOWM5THJtN3NIREtHQ0Rxd09ZSEtJZUxnb2J2VUtQV3hGQTBQMThzYjVGUkx0ZHpkS2s3UFVfUzYtdTNHSHNuak91VkVqSnlzS0x5T1RQY3BoT2ktbzZpazB5MnBYNUwxakpsS1NxSFRvemdSby1n?oc=5）</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="180" customHeight="1" s="2">
+          <t>利多：劳动力短缺可能拖慢收割和入榨节奏，减少短期可用糖源。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="179.1" customHeight="1" s="2">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>斐济</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 Soko Directory报道：A Look At Prices Of Sugar Across Naivas, Cleanshelf, Quickmart And Carrefour。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
+          <t>FBC News称，斐济蔗农获得成本缓解支持，有助于降低种植和收割环节的现金压力。成本压力缓和有利于维持甘蔗供应和农户种植积极性，对中长期供应偏利空。来源：FBC News（https://news.google.com/rss/articles/CBMibkFVX3lxTE1tSk9tQ3ZYajFRT0tuZTZBdTBKdTFaMEVwaC1hdWFmdjRtZGx4THJPVGZvNEozWW1oVzIxUUVBWlZBVWNwcWlhV0RqOXNnMHkzN2E5bmV3MkZfek0tbkxYcGNuUVc4eEE4Uk9nSERn?oc=5）</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：成本压力缓和有助于稳定甘蔗生产和未来供应。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="180" customHeight="1" s="2">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>肯尼亚</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 Latin Lawyer报道：Raízen sells sugar mill to Adecoagro amid restructuring。来源：Latin Lawyer（https://news.google.com/rss/articles/CBMijAFBVV95cUxPeWNVcmtMWnhqV3FzUTlma1BBUjdvdmY3MEE2cURqUEJwZVdKN2NZbnpCQk01MXlueEZVczdzS0VveDFielZQVHFlbFFkTlNYOEMwbm92VGt5SHhrR3lGSDYySGtocGJTM09YTnc5YmtVV0JmZWNLd1NDQ1ZpNmFURld5UTVSLWp5VWFXOA?oc=5）</t>
+          <t>Soko Directory对肯尼亚 Naivas、Cleanshelf、Quickmart 和 Carrefour 等零售渠道食糖价格进行比较。零售价格信息反映终端消费成本和渠道供应情况，但对区域产量和贸易流向的直接影响有限。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：零售价格信息主要反映终端成本，暂未改变供应判断。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="180" customHeight="1" s="2">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>南非</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 African Farming报道：Sugar industry under pressure as foreign cane cutters flee violence。来源：African Farming（https://news.google.com/rss/articles/CBMirwFBVV95cUxNZnNSU0Q3eUU0S2ljeUV4LUVoZ3ZKRGowci1CN1VGRDN0MG13NEl4Z3BkWjEteVJabnY2ZEhUc3IySkU5blpHN1JDN0J3S3plNDlMMnl1XzRZRTF5bVZET2lEbmRVUE51cWNqcWdwazhCaF9sRERIQkl6S0FoTXhSdEo4WFg5aHNtckJWN09HUTcyNXowVU54MjdGQUdnVkxaZ25IQk95MzlGWkRseGVj?oc=5）</t>
+          <t>African Farming称，外籍砍蔗工因暴力事件离开，南非相关糖业生产面临劳动力压力。若劳动力短缺持续，甘蔗收割和糖厂入榨节奏可能受阻，减少短期可用供应。来源：African Farming（https://news.google.com/rss/articles/CBMirwFBVV95cUxNZnNSU0Q3eUU0S2ljeUV4LUVoZ3ZKRGowci1CN1VGRDN0MG13NEl4Z3BkWjEteVJabnY2ZEhUc3IySkU5blpHN1JDN0J3S3plNDlMMnl1XzRZRTF5bVZET2lEbmRVUE51cWNqcWdwazhCaF9sRERIQkl6S0FoTXhSdEo4WFg5aHNtckJWN09HUTcyNXowVU54MjdGQUdnVkxaZ25IQk95MzlGWkRseGVj?oc=5）</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="180" customHeight="1" s="2">
+          <t>利多：劳动力扰动可能拖慢甘蔗收割和压榨节奏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="161.5" customHeight="1" s="2">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>菲律宾</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 Inquirer.net报道：Negros small sugar farmers to get cash aid amid pest outbreak。来源：Inquirer.net（https://news.google.com/rss/articles/CBMioAFBVV95cUxOckMxNTNFTmN5NUdFNjF5ZWlFbnJCTUxwdWlsNTBhcmNGQkZTRnRkZTJCOFlxNjVKWTU5MTVkeXo1N0NKUjVYbkJSbEdQdUdGQzFOaW9iX1kwdHhGa0d5dUJfRTNqZVRmY2JKZndZbHRrdWVXbVcxV0w1UjBoWjBtQWNLSktEZ0FZRUVNMkliM01TUHRiU2kyQ2pkSl9GUjdw0gGmAUFVX3lxTE5Na1Z5Qzc5VGFZWC1ZQzdKX0dFRUZLbUxfM29kNlczU0g1ejFuQjFseDB5QmpFOXNNV1lyRFVGU0kyOU9XLWxsNl8wazY4TXlKcG5MaWgxQ2RhXzgxRUplZUxCd0VXSmw4LUNRck01cXVydnczMExEYlFhZk9uTEkxVExYaTBQd0szQXpiRTF2ZC1lUkZfLXRFaWMwdEh0SGpEOHM4d2c?oc=5）</t>
+          <t>pna.gov.ph称，菲律宾 Negros 受甘蔗虫害影响的蔗农有望获得现金援助。病虫害已对甘蔗生产形成压力，补助有助于缓解农户现金流，但难以立即修复作物损失。来源：pna.gov.ph（https://news.google.com/rss/articles/CBMiUEFVX3lxTE45d0EzQU1WZ3NkakdIT0t6X3pMOE5OT09nVVpoZG5Ib0pvMWNTemFJMFhyYjhObUdwcjlnb3F0UWQ2MnVTV0puZEFnUTZMLTND?oc=5）</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="167" customHeight="1" s="2">
+          <t>利多：虫害损失可能削弱当地甘蔗供应，现金援助难以立即恢复产量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="162.05" customHeight="1" s="2">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>孟加拉国</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 pna.gov.ph报道：DSWD eyes cash assistance for sugarcane pest-hit farmers in Negros。来源：pna.gov.ph（https://news.google.com/rss/articles/CBMiUEFVX3lxTE45d0EzQU1WZ3NkakdIT0t6X3pMOE5OT09nVVpoZG5Ib0pvMWNTemFJMFhyYjhObUdwcjlnb3F0UWQ2MnVTV0puZEFnUTZMLTND?oc=5）</t>
+          <t>Daily Observer称，孟加拉国 Tangail 甘蔗遭病毒侵袭并造成作物受损，蔗农生产积极性受到影响。病害导致糖料供应受损风险上升，对当地食糖生产预期偏利多糖价。来源：Daily Observer（https://news.google.com/rss/articles/CBMiSkFVX3lxTE94WnJDZnpNNlJKOHdEeWcyTkFNc2ZCTHYtZFcxZHdqR1Y2QmlUeTltcE9EaWpCTGRfQ3J0WURjb05DREtXTTVMSkpn?oc=5）</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利多：病害损害甘蔗作物，可能减少当地糖料供应。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="180" customHeight="1" s="2">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>其他国家</t>
+          <t>菲律宾</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 SME Futures报道：Allahabad HC seeks accountability in two-decade-old sugarcane dues case。来源：SME Futures（https://news.google.com/rss/articles/CBMimwFBVV95cUxPcWRaX2lqME5GZ042V092SzAyZXByMjI2N2F2R3o1bmUzUkRXSU5VOC1YYkh2MmFmQUJVTDRnN2c3WWlra21xdTlMT2M1WDJqZElKWmFHY1JkNGFMcDQteXNZOWotSjY1MThJMnVLNFE1SG0zQ1p2WktoRjVubXVsVlBCSXprLUFmYzRNbHJJOGRfd2pvaE5GTGgzNA?oc=5）</t>
+          <t>Panay News称，菲律宾 Negros Occidental 启动甘蔗病虫害生物防治行动。防治措施有助于降低虫害继续扩散风险，稳定当地糖料供应预期。来源：Panay News（https://news.google.com/rss/articles/CBMiiwFBVV95cUxQYTgyYmxUSmFjYXI4Tkx2MDFYTm93eWtSV2ZsNEt0Y0V0WlVkdFBGVzlSNVE1M2JPVEJaUlNuYWpjRTZKV0xpN1dQcm4tM0lPOVZ3bVlGWXcwVkRjVVNxNHRPX3NWZHFDT1JsZzI2ZVB6UVJydlB5RThNVXUza1I1dmdWOWVVY0ktY3g0?oc=5）</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="167" customHeight="1" s="2">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-23 Daily Observer报道：Sugarcane farmers frustrated as virus attack ruins crop in Tangail。来源：Daily Observer（https://news.google.com/rss/articles/CBMiSkFVX3lxTE94WnJDZnpNNlJKOHdEeWcyTkFNc2ZCTHYtZFcxZHdqR1Y2QmlUeTltcE9EaWpCTGRfQ3J0WURjb05DREtXTTVMSkpn?oc=5）</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="180" customHeight="1" s="2">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-23 Panay News报道：NegOcc begins biological control drive vs sugarcane pest。来源：Panay News（https://news.google.com/rss/articles/CBMiiwFBVV95cUxQYTgyYmxUSmFjYXI4Tkx2MDFYTm93eWtSV2ZsNEt0Y0V0WlVkdFBGVzlSNVE1M2JPVEJaUlNuYWpjRTZKV0xpN1dQcm4tM0lPOVZ3bVlGWXcwVkRjVVNxNHRPX3NWZHFDT1JsZzI2ZVB6UVJydlB5RThNVXUza1I1dmdWOWVVY0ktY3g0?oc=5）</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：病虫害防控推进有助于降低后续产量损失风险。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add mandatory Thailand cane rainfall news check
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-23.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-23.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -627,117 +627,134 @@
     <row r="9" ht="180" customHeight="1" s="2">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>泰国</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Open-Meteo预报显示（2026-07-24至2026-07-30），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括甘烹碧约169.0mm、沙缴约163.6mm、加拉信约131.2mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="180" customHeight="1" s="2">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>斐济</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>FBC News称，斐济糖业部门面临劳动力短缺压力，甘蔗收割和糖厂运行可能受到影响。若砍蔗工供应不足持续，甘蔗入榨节奏和当季产量释放可能放慢。来源：FBC News（https://news.google.com/rss/articles/CBMid0FVX3lxTE9IOWM5THJtN3NIREtHQ0Rxd09ZSEtJZUxnb2J2VUtQV3hGQTBQMThzYjVGUkx0ZHpkS2s3UFVfUzYtdTNHSHNuak91VkVqSnlzS0x5T1RQY3BoT2ktbzZpazB5MnBYNUwxakpsS1NxSFRvemdSby1n?oc=5）</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>利多：劳动力短缺可能拖慢收割和入榨节奏，减少短期可用糖源。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="179.1" customHeight="1" s="2">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11" ht="179.1" customHeight="1" s="2">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>斐济</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>FBC News称，斐济蔗农获得成本缓解支持，有助于降低种植和收割环节的现金压力。成本压力缓和有利于维持甘蔗供应和农户种植积极性，对中长期供应偏利空。来源：FBC News（https://news.google.com/rss/articles/CBMibkFVX3lxTE1tSk9tQ3ZYajFRT0tuZTZBdTBKdTFaMEVwaC1hdWFmdjRtZGx4THJPVGZvNEozWW1oVzIxUUVBWlZBVWNwcWlhV0RqOXNnMHkzN2E5bmV3MkZfek0tbkxYcGNuUVc4eEE4Uk9nSERn?oc=5）</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>利空：成本压力缓和有助于稳定甘蔗生产和未来供应。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="180" customHeight="1" s="2">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>肯尼亚</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Soko Directory对肯尼亚 Naivas、Cleanshelf、Quickmart 和 Carrefour 等零售渠道食糖价格进行比较。零售价格信息反映终端消费成本和渠道供应情况，但对区域产量和贸易流向的直接影响有限。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>中性：零售价格信息主要反映终端成本，暂未改变供应判断。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="180" customHeight="1" s="2">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>肯尼亚</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Soko Directory对肯尼亚 Naivas、Cleanshelf、Quickmart 和 Carrefour 等零售渠道食糖价格进行比较。零售价格信息反映终端消费成本和渠道供应情况，但对区域产量和贸易流向的直接影响有限。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>中性：零售价格信息主要反映终端成本，暂未改变供应判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="180" customHeight="1" s="2">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>南非</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>African Farming称，外籍砍蔗工因暴力事件离开，南非相关糖业生产面临劳动力压力。若劳动力短缺持续，甘蔗收割和糖厂入榨节奏可能受阻，减少短期可用供应。来源：African Farming（https://news.google.com/rss/articles/CBMirwFBVV95cUxNZnNSU0Q3eUU0S2ljeUV4LUVoZ3ZKRGowci1CN1VGRDN0MG13NEl4Z3BkWjEteVJabnY2ZEhUc3IySkU5blpHN1JDN0J3S3plNDlMMnl1XzRZRTF5bVZET2lEbmRVUE51cWNqcWdwazhCaF9sRERIQkl6S0FoTXhSdEo4WFg5aHNtckJWN09HUTcyNXowVU54MjdGQUdnVkxaZ25IQk95MzlGWkRseGVj?oc=5）</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>利多：劳动力扰动可能拖慢甘蔗收割和压榨节奏。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="161.5" customHeight="1" s="2">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14" ht="161.5" customHeight="1" s="2">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>菲律宾</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>pna.gov.ph称，菲律宾 Negros 受甘蔗虫害影响的蔗农有望获得现金援助。病虫害已对甘蔗生产形成压力，补助有助于缓解农户现金流，但难以立即修复作物损失。来源：pna.gov.ph（https://news.google.com/rss/articles/CBMiUEFVX3lxTE45d0EzQU1WZ3NkakdIT0t6X3pMOE5OT09nVVpoZG5Ib0pvMWNTemFJMFhyYjhObUdwcjlnb3F0UWQ2MnVTV0puZEFnUTZMLTND?oc=5）</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>利多：虫害损失可能削弱当地甘蔗供应，现金援助难以立即恢复产量。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="162.05" customHeight="1" s="2">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="162.05" customHeight="1" s="2">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>孟加拉国</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Daily Observer称，孟加拉国 Tangail 甘蔗遭病毒侵袭并造成作物受损，蔗农生产积极性受到影响。病害导致糖料供应受损风险上升，对当地食糖生产预期偏利多糖价。来源：Daily Observer（https://news.google.com/rss/articles/CBMiSkFVX3lxTE94WnJDZnpNNlJKOHdEeWcyTkFNc2ZCTHYtZFcxZHdqR1Y2QmlUeTltcE9EaWpCTGRfQ3J0WURjb05DREtXTTVMSkpn?oc=5）</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>利多：病害损害甘蔗作物，可能减少当地糖料供应。</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="180" customHeight="1" s="2">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="180" customHeight="1" s="2">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>菲律宾</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Panay News称，菲律宾 Negros Occidental 启动甘蔗病虫害生物防治行动。防治措施有助于降低虫害继续扩散风险，稳定当地糖料供应预期。来源：Panay News（https://news.google.com/rss/articles/CBMiiwFBVV95cUxQYTgyYmxUSmFjYXI4Tkx2MDFYTm93eWtSV2ZsNEt0Y0V0WlVkdFBGVzlSNVE1M2JPVEJaUlNuYWpjRTZKV0xpN1dQcm4tM0lPOVZ3bVlGWXcwVkRjVVNxNHRPX3NWZHFDT1JsZzI2ZVB6UVJydlB5RThNVXUza1I1dmdWOWVVY0ktY3g0?oc=5）</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>利空：病虫害防控推进有助于降低后续产量损失风险。</t>
         </is>

</xml_diff>

<commit_message>
Add China Sugar News monitoring and items
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-23.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-23.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -641,120 +641,188 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="180" customHeight="1" s="2">
+    <row r="10" ht="117.5" customHeight="1" s="2">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2015—2025年中国进口甘蔗由105.41万吨增至359.07万吨，十年增长约240.6%；2026年1—6月累计进口326.12万吨，已相当于2025年全年的90.8%。进口甘蔗持续补充国内糖料供应，有利于提高边境糖厂原料保障，对国内糖价形成偏空影响。来源：云糖网（https://www.yntw.com/date/2026/07）</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>利空：进口甘蔗快速增长增加国内糖料补充，改善边境糖厂原料保障并提高后续供给预期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="123.55" customHeight="1" s="2">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>国内食糖工业库存约449万吨，仍处于历史同期偏高水平；6月进口食糖28万吨，市场预计7月以后进口量继续增加。高库存叠加进口到港增长，将继续压制国内现货及郑糖价格的反弹空间。来源：紫金天风期货（https://finance.sina.com.cn/money/future/fmnews/2026-07-23/doc-iniiusky8326649.shtml）</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>利空：库存高位和进口增加共同抬升国内可用供应，限制现货及郑糖价格上行空间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="116.95" customHeight="1" s="2">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>广西制糖集团报价维持5170—5270元/吨，云南制糖集团报价4980—5030元/吨、部分下调10元/吨，加工糖报价总体稳定。现货需求没有明显改善，国内市场缺少新的上涨驱动，短期糖价预计维持低位震荡。来源：光大期货市场观点（https://goodsfu.10jqka.com.cn/20260723/c678373891.shtml）</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>中性：现货购销平稳但需求改善不足，云南小幅下调报价显示价格上行动能偏弱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="116.95" customHeight="1" s="2">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>7月23日夜间起，云南文山、红河、玉溪、普洱等甘蔗产区有中到大雨、局部暴雨至大暴雨预报，部分地区伴有短时强降水、大风和冰雹。强降雨可能造成局部农田积水、甘蔗倒伏及田间管理困难，短期对甘蔗生长和后续供应存在不利影响。来源：云南网（https://yn.yunnan.cn/system/2026/07/24/034094070.shtml）</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>利多：云南甘蔗产区强降雨可能引发积水、倒伏和田间管理困难，短期削弱糖料供应稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="180" customHeight="1" s="2">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>斐济</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>FBC News称，斐济糖业部门面临劳动力短缺压力，甘蔗收割和糖厂运行可能受到影响。若砍蔗工供应不足持续，甘蔗入榨节奏和当季产量释放可能放慢。来源：FBC News（https://news.google.com/rss/articles/CBMid0FVX3lxTE9IOWM5THJtN3NIREtHQ0Rxd09ZSEtJZUxnb2J2VUtQV3hGQTBQMThzYjVGUkx0ZHpkS2s3UFVfUzYtdTNHSHNuak91VkVqSnlzS0x5T1RQY3BoT2ktbzZpazB5MnBYNUwxakpsS1NxSFRvemdSby1n?oc=5）</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>利多：劳动力短缺可能拖慢收割和入榨节奏，减少短期可用糖源。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="179.1" customHeight="1" s="2">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="15" ht="179.1" customHeight="1" s="2">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>斐济</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>FBC News称，斐济蔗农获得成本缓解支持，有助于降低种植和收割环节的现金压力。成本压力缓和有利于维持甘蔗供应和农户种植积极性，对中长期供应偏利空。来源：FBC News（https://news.google.com/rss/articles/CBMibkFVX3lxTE1tSk9tQ3ZYajFRT0tuZTZBdTBKdTFaMEVwaC1hdWFmdjRtZGx4THJPVGZvNEozWW1oVzIxUUVBWlZBVWNwcWlhV0RqOXNnMHkzN2E5bmV3MkZfek0tbkxYcGNuUVc4eEE4Uk9nSERn?oc=5）</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>利空：成本压力缓和有助于稳定甘蔗生产和未来供应。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="180" customHeight="1" s="2">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>肯尼亚</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Soko Directory对肯尼亚 Naivas、Cleanshelf、Quickmart 和 Carrefour 等零售渠道食糖价格进行比较。零售价格信息反映终端消费成本和渠道供应情况，但对区域产量和贸易流向的直接影响有限。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>中性：零售价格信息主要反映终端成本，暂未改变供应判断。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="180" customHeight="1" s="2">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>南非</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>African Farming称，外籍砍蔗工因暴力事件离开，南非相关糖业生产面临劳动力压力。若劳动力短缺持续，甘蔗收割和糖厂入榨节奏可能受阻，减少短期可用供应。来源：African Farming（https://news.google.com/rss/articles/CBMirwFBVV95cUxNZnNSU0Q3eUU0S2ljeUV4LUVoZ3ZKRGowci1CN1VGRDN0MG13NEl4Z3BkWjEteVJabnY2ZEhUc3IySkU5blpHN1JDN0J3S3plNDlMMnl1XzRZRTF5bVZET2lEbmRVUE51cWNqcWdwazhCaF9sRERIQkl6S0FoTXhSdEo4WFg5aHNtckJWN09HUTcyNXowVU54MjdGQUdnVkxaZ25IQk95MzlGWkRseGVj?oc=5）</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>利多：劳动力扰动可能拖慢甘蔗收割和压榨节奏。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="161.5" customHeight="1" s="2">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>pna.gov.ph称，菲律宾 Negros 受甘蔗虫害影响的蔗农有望获得现金援助。病虫害已对甘蔗生产形成压力，补助有助于缓解农户现金流，但难以立即修复作物损失。来源：pna.gov.ph（https://news.google.com/rss/articles/CBMiUEFVX3lxTE45d0EzQU1WZ3NkakdIT0t6X3pMOE5OT09nVVpoZG5Ib0pvMWNTemFJMFhyYjhObUdwcjlnb3F0UWQ2MnVTV0puZEFnUTZMLTND?oc=5）</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>利多：虫害损失可能削弱当地甘蔗供应，现金援助难以立即恢复产量。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="162.05" customHeight="1" s="2">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>孟加拉国</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Daily Observer称，孟加拉国 Tangail 甘蔗遭病毒侵袭并造成作物受损，蔗农生产积极性受到影响。病害导致糖料供应受损风险上升，对当地食糖生产预期偏利多糖价。来源：Daily Observer（https://news.google.com/rss/articles/CBMiSkFVX3lxTE94WnJDZnpNNlJKOHdEeWcyTkFNc2ZCTHYtZFcxZHdqR1Y2QmlUeTltcE9EaWpCTGRfQ3J0WURjb05DREtXTTVMSkpn?oc=5）</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>利多：病害损害甘蔗作物，可能减少当地糖料供应。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="180" customHeight="1" s="2">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>肯尼亚</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Soko Directory对肯尼亚 Naivas、Cleanshelf、Quickmart 和 Carrefour 等零售渠道食糖价格进行比较。零售价格信息反映终端消费成本和渠道供应情况，但对区域产量和贸易流向的直接影响有限。来源：Soko Directory（https://news.google.com/rss/articles/CBMirgFBVV95cUxOdUhzclpzOUg1eXMyeWV5eElJNS0zeUhQelk3RlU2aHEtR1g2Z0NGMy1MN0E0aGRQMWdWbmNqcTBRLWp6TzJ1bFN4U1BlZXNVMDBYVDhzb2U2cU1IUjJhcW41bEJ0UE1jNmNnWl9WcmFDTU5DaHA4WUwtd0RqMnhtc25YTTZrQmw0RmstQnZ0UWhTTEsyLVlZT2hMY3lRdm1Nb1RzQnpXNEVEaDY2VHfSAbMBQVVfeXFMTVJmTmc4X3NvU1JsbDVvYTFwY1UzWXJUYW1HYVZic0dzXzJselhmZHhzZHRfUGVzSTUya0dmZEVtYzFOaEdsNU5ONU5qY050TlhCRFJicVhNZWw2UFVzMG5OYl9tVE5Mdkk3R2FqNXBWOXg3STZBdXBrLUdXR09kZDVuRHoyQjZ5SkRockNmdG5iZEVqV1gwVExwSHRjY3NvRWZpSXZxMElWbWhmd2dDWGdRMEE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>中性：零售价格信息主要反映终端成本，暂未改变供应判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="180" customHeight="1" s="2">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>南非</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>African Farming称，外籍砍蔗工因暴力事件离开，南非相关糖业生产面临劳动力压力。若劳动力短缺持续，甘蔗收割和糖厂入榨节奏可能受阻，减少短期可用供应。来源：African Farming（https://news.google.com/rss/articles/CBMirwFBVV95cUxNZnNSU0Q3eUU0S2ljeUV4LUVoZ3ZKRGowci1CN1VGRDN0MG13NEl4Z3BkWjEteVJabnY2ZEhUc3IySkU5blpHN1JDN0J3S3plNDlMMnl1XzRZRTF5bVZET2lEbmRVUE51cWNqcWdwazhCaF9sRERIQkl6S0FoTXhSdEo4WFg5aHNtckJWN09HUTcyNXowVU54MjdGQUdnVkxaZ25IQk95MzlGWkRseGVj?oc=5）</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>利多：劳动力扰动可能拖慢甘蔗收割和压榨节奏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="161.5" customHeight="1" s="2">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>菲律宾</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>pna.gov.ph称，菲律宾 Negros 受甘蔗虫害影响的蔗农有望获得现金援助。病虫害已对甘蔗生产形成压力，补助有助于缓解农户现金流，但难以立即修复作物损失。来源：pna.gov.ph（https://news.google.com/rss/articles/CBMiUEFVX3lxTE45d0EzQU1WZ3NkakdIT0t6X3pMOE5OT09nVVpoZG5Ib0pvMWNTemFJMFhyYjhObUdwcjlnb3F0UWQ2MnVTV0puZEFnUTZMLTND?oc=5）</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>利多：虫害损失可能削弱当地甘蔗供应，现金援助难以立即恢复产量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="162.05" customHeight="1" s="2">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>孟加拉国</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Daily Observer称，孟加拉国 Tangail 甘蔗遭病毒侵袭并造成作物受损，蔗农生产积极性受到影响。病害导致糖料供应受损风险上升，对当地食糖生产预期偏利多糖价。来源：Daily Observer（https://news.google.com/rss/articles/CBMiSkFVX3lxTE94WnJDZnpNNlJKOHdEeWcyTkFNc2ZCTHYtZFcxZHdqR1Y2QmlUeTltcE9EaWpCTGRfQ3J0WURjb05DREtXTTVMSkpn?oc=5）</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>利多：病害损害甘蔗作物，可能减少当地糖料供应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="180" customHeight="1" s="2">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Panay News称，菲律宾 Negros Occidental 启动甘蔗病虫害生物防治行动。防治措施有助于降低虫害继续扩散风险，稳定当地糖料供应预期。来源：Panay News（https://news.google.com/rss/articles/CBMiiwFBVV95cUxQYTgyYmxUSmFjYXI4Tkx2MDFYTm93eWtSV2ZsNEt0Y0V0WlVkdFBGVzlSNVE1M2JPVEJaUlNuYWpjRTZKV0xpN1dQcm4tM0lPOVZ3bVlGWXcwVkRjVVNxNHRPX3NWZHFDT1JsZzI2ZVB6UVJydlB5RThNVXUza1I1dmdWOWVVY0ktY3g0?oc=5）</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>利空：病虫害防控推进有助于降低后续产量损失风险。</t>
         </is>

</xml_diff>